<commit_message>
docs(roi): update executive dashboard source workbook values
</commit_message>
<xml_diff>
--- a/ROI.xlsx
+++ b/ROI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikhil/Documents/ECS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC786EF6-B56E-7E4E-9ECA-7088BC177E1F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1B385D-2B1F-404D-9EA2-77193F829CA3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FY 25 -26" sheetId="6" r:id="rId1"/>
@@ -22,42 +22,6 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FY 25 -26'!$A$1:$L$18</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">Executive_Dashboard!$A$2</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Executive_Dashboard!$A$3</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">Executive_Dashboard!$A$2</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">Executive_Dashboard!$A$3</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Executive_Dashboard!$A$4</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">Executive_Dashboard!$A$4</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">Executive_Dashboard!$A$5</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">Executive_Dashboard!$B$1:$H$1</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">Executive_Dashboard!$B$2:$H$2</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">Executive_Dashboard!$B$3:$H$3</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">Executive_Dashboard!$B$4:$H$4</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">Executive_Dashboard!$B$5:$H$5</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">Executive_Dashboard!$A$2</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">Executive_Dashboard!$A$3</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">Executive_Dashboard!$A$4</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Executive_Dashboard!$A$5</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">Executive_Dashboard!$A$5</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">Executive_Dashboard!$B$1:$H$1</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">Executive_Dashboard!$B$2:$H$2</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">Executive_Dashboard!$B$3:$H$3</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">Executive_Dashboard!$B$4:$H$4</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">Executive_Dashboard!$B$5:$H$5</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Executive_Dashboard!$B$1:$H$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Executive_Dashboard!$B$2:$H$2</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Executive_Dashboard!$B$3:$H$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Executive_Dashboard!$B$4:$H$4</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Executive_Dashboard!$B$5:$H$5</definedName>
-    <definedName name="_xlchart.v2.10" hidden="1">Executive_Dashboard!$A$3</definedName>
-    <definedName name="_xlchart.v2.11" hidden="1">Executive_Dashboard!$A$4</definedName>
-    <definedName name="_xlchart.v2.12" hidden="1">Executive_Dashboard!$A$5</definedName>
-    <definedName name="_xlchart.v2.13" hidden="1">Executive_Dashboard!$B$1:$H$1</definedName>
-    <definedName name="_xlchart.v2.14" hidden="1">Executive_Dashboard!$B$2:$H$2</definedName>
-    <definedName name="_xlchart.v2.15" hidden="1">Executive_Dashboard!$B$3:$H$3</definedName>
-    <definedName name="_xlchart.v2.16" hidden="1">Executive_Dashboard!$B$4:$H$4</definedName>
-    <definedName name="_xlchart.v2.17" hidden="1">Executive_Dashboard!$B$5:$H$5</definedName>
-    <definedName name="_xlchart.v2.9" hidden="1">Executive_Dashboard!$A$2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -656,7 +620,7 @@
                   <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>400</c:v>
+                  <c:v>600</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>800</c:v>
@@ -745,7 +709,7 @@
                   <c:v>90.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>72.64</c:v>
+                  <c:v>108.96000000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>145.28</c:v>
@@ -923,7 +887,7 @@
                   <c:v>88.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>70.44</c:v>
+                  <c:v>106.76</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>143.08000000000001</c:v>
@@ -3892,7 +3856,7 @@
         <v>500</v>
       </c>
       <c r="G2" s="2">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="H2" s="2">
         <v>800</v>
@@ -3922,8 +3886,8 @@
         <v>90.8</v>
       </c>
       <c r="G3" s="2">
-        <f>C3*4</f>
-        <v>72.64</v>
+        <f>C3*6</f>
+        <v>108.96000000000001</v>
       </c>
       <c r="H3" s="2">
         <f>C3*8</f>
@@ -3982,7 +3946,7 @@
       </c>
       <c r="G5" s="2">
         <f>G3-G4</f>
-        <v>70.44</v>
+        <v>106.76</v>
       </c>
       <c r="H5" s="2">
         <f>H3-H4</f>
@@ -4009,14 +3973,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="f9ef682c-7912-4780-84f4-a971df966cba" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b405d1f-d10b-4093-82f9-1855360715f6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4221,21 +4183,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="f9ef682c-7912-4780-84f4-a971df966cba" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7b405d1f-d10b-4093-82f9-1855360715f6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF0D1079-5B4B-49D4-ADDA-486E009CBEBA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20FF6A95-94CC-4354-9C77-CD818EDE354A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f9ef682c-7912-4780-84f4-a971df966cba"/>
-    <ds:schemaRef ds:uri="7b405d1f-d10b-4093-82f9-1855360715f6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4260,9 +4221,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20FF6A95-94CC-4354-9C77-CD818EDE354A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF0D1079-5B4B-49D4-ADDA-486E009CBEBA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f9ef682c-7912-4780-84f4-a971df966cba"/>
+    <ds:schemaRef ds:uri="7b405d1f-d10b-4093-82f9-1855360715f6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>